<commit_message>
Docs: wrong-plug check and errata list, component list and supplier quote request (rev 5 design, one servo type), costing notes, Alibaba quote request (part 1 of 2)
</commit_message>
<xml_diff>
--- a/docs/RoboCore_V2_component_list.xlsx
+++ b/docs/RoboCore_V2_component_list.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Component list'!$A$7:$R$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Component list'!$A$7:$R$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Component list'!$7:$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -354,34 +354,49 @@
         <t>MG90D shown (Adafruit's metal-gear micro servo). The MG90S is the same size, horns and mounting.</t>
       </text>
     </comment>
-    <comment ref="C18" authorId="1" shapeId="0">
+    <comment ref="C17" authorId="1" shapeId="0">
       <text>
         <t>Shown: 3- and 4-cell holders. Buy a 3 × 18650 holder (about 61.6 × 78.4 mm) and wire it in PARALLEL (1S3P).</t>
       </text>
     </comment>
-    <comment ref="C19" authorId="1" shapeId="0">
-      <text>
-        <t>Similar, not the same: a TP4056 charger board whose right half (DW01 + 8205A, B+/B−/OUT+/OUT−) is the protection circuit. Buy the protection-only board; the controller already charges the battery.</t>
-      </text>
-    </comment>
-    <comment ref="C20" authorId="1" shapeId="0">
+    <comment ref="C18" authorId="1" shapeId="0">
       <text>
         <t>Board side shown: the male XT30 on the controller. Buy the FEMALE XT30U-F with leads, which plugs into it.</t>
       </text>
     </comment>
-    <comment ref="C25" authorId="1" shapeId="0">
+    <comment ref="C21" authorId="1" shapeId="0">
       <text>
         <t>Any 5 V, 2 A USB charger will do.</t>
       </text>
     </comment>
-    <comment ref="C27" authorId="1" shapeId="0">
+    <comment ref="C23" authorId="1" shapeId="0">
       <text>
         <t>M3 × 4 inserts shown; the M2 ones look the same, only smaller.</t>
       </text>
     </comment>
+    <comment ref="C24" authorId="1" shapeId="0">
+      <text>
+        <t>M3 × 4 brass heat-set inserts (Adafruit 4255).</t>
+      </text>
+    </comment>
+    <comment ref="C25" authorId="1" shapeId="0">
+      <text>
+        <t>Phillips pan head machine screw (not to scale).</t>
+      </text>
+    </comment>
+    <comment ref="C26" authorId="1" shapeId="0">
+      <text>
+        <t>Self-tapping screws (not to scale); pan head wanted.</t>
+      </text>
+    </comment>
+    <comment ref="C27" authorId="1" shapeId="0">
+      <text>
+        <t>Flat washers (not to scale).</t>
+      </text>
+    </comment>
     <comment ref="C28" authorId="1" shapeId="0">
       <text>
-        <t>M3 × 4 brass heat-set inserts (Adafruit 4255).</t>
+        <t>Phillips pan head machine screw (not to scale).</t>
       </text>
     </comment>
     <comment ref="C29" authorId="1" shapeId="0">
@@ -391,75 +406,55 @@
     </comment>
     <comment ref="C30" authorId="1" shapeId="0">
       <text>
-        <t>Self-tapping screws (not to scale); pan head wanted.</t>
+        <t>Phillips pan head machine screw (not to scale).</t>
       </text>
     </comment>
     <comment ref="C31" authorId="1" shapeId="0">
       <text>
-        <t>Flat washers (not to scale).</t>
+        <t>Socket head cap screw (not to scale).</t>
       </text>
     </comment>
     <comment ref="C32" authorId="1" shapeId="0">
       <text>
-        <t>Phillips pan head machine screw (not to scale).</t>
+        <t>Self-tapping screws (not to scale); pan head wanted.</t>
       </text>
     </comment>
     <comment ref="C33" authorId="1" shapeId="0">
       <text>
-        <t>Phillips pan head machine screw (not to scale).</t>
+        <t>Star-knob thumb screw shown; the list asks for a knurled-head M3 × 8 thumb screw.</t>
       </text>
     </comment>
     <comment ref="C34" authorId="1" shapeId="0">
       <text>
-        <t>Phillips pan head machine screw (not to scale).</t>
+        <t>Hex nuts on a bolt (not to scale): plain M8 hex nuts.</t>
       </text>
     </comment>
     <comment ref="C35" authorId="1" shapeId="0">
       <text>
-        <t>Socket head cap screw (not to scale).</t>
-      </text>
-    </comment>
-    <comment ref="C36" authorId="1" shapeId="0">
-      <text>
-        <t>Self-tapping screws (not to scale); pan head wanted.</t>
+        <t>Polished steel ball, shown much bigger than life: you need ½" (12.7 mm) balls.</t>
       </text>
     </comment>
     <comment ref="C37" authorId="1" shapeId="0">
       <text>
-        <t>Star-knob thumb screw shown; the list asks for a knurled-head M3 × 8 thumb screw.</t>
+        <t>Filament spools (generic photo). Buy PETG in the colour on this line.</t>
       </text>
     </comment>
     <comment ref="C38" authorId="1" shapeId="0">
       <text>
-        <t>Hex nuts on a bolt (not to scale): plain M8 hex nuts.</t>
+        <t>Filament spools (generic photo). Buy black PETG.</t>
       </text>
     </comment>
     <comment ref="C39" authorId="1" shapeId="0">
       <text>
-        <t>Polished steel ball, shown much bigger than life: you need ½" (12.7 mm) balls.</t>
-      </text>
-    </comment>
-    <comment ref="C41" authorId="1" shapeId="0">
-      <text>
-        <t>Filament spools (generic photo). Buy PETG in the colour on this line.</t>
-      </text>
-    </comment>
-    <comment ref="C42" authorId="1" shapeId="0">
-      <text>
-        <t>Filament spools (generic photo). Buy black PETG.</t>
-      </text>
-    </comment>
-    <comment ref="C43" authorId="1" shapeId="0">
-      <text>
         <t>Filament spools (generic photo). Buy dark teal PETG.</t>
       </text>
     </comment>
-    <comment ref="C44" authorId="1" shapeId="0">
+    <comment ref="C40" authorId="1" shapeId="0">
       <text>
         <t>Filament spools (generic photo). Buy black TPU 95A.</t>
       </text>
     </comment>
-    <comment ref="C51" authorId="1" shapeId="0">
+    <comment ref="C47" authorId="1" shapeId="0">
       <text>
         <t>M3 heat-set insert tip shown; get the M2 tip as well, to fit your iron.</t>
       </text>
@@ -506,6 +501,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -531,6 +529,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -556,6 +557,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -581,6 +585,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -606,6 +613,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -614,13 +624,13 @@
     <from>
       <col>2</col>
       <colOff>66675</colOff>
-      <row>14</row>
-      <rowOff>114300</rowOff>
+      <row>15</row>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="1143000" cy="704850"/>
+    <ext cx="1143000" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -631,6 +641,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -640,12 +653,12 @@
       <col>2</col>
       <colOff>66675</colOff>
       <row>16</row>
-      <rowOff>38100</rowOff>
+      <rowOff>85725</rowOff>
     </from>
-    <ext cx="1143000" cy="857250"/>
+    <ext cx="1143000" cy="762000"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -656,6 +669,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -663,14 +679,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>66675</colOff>
+      <colOff>95250</colOff>
       <row>17</row>
-      <rowOff>85725</rowOff>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="1143000" cy="762000"/>
+    <ext cx="1085850" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -681,6 +697,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -688,14 +707,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>161925</colOff>
-      <row>18</row>
-      <rowOff>161925</rowOff>
+      <colOff>76200</colOff>
+      <row>19</row>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="952500" cy="609600"/>
+    <ext cx="1114425" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -706,6 +725,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -713,14 +735,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>95250</colOff>
-      <row>19</row>
-      <rowOff>38100</rowOff>
+      <colOff>66675</colOff>
+      <row>20</row>
+      <rowOff>76200</rowOff>
     </from>
-    <ext cx="1085850" cy="857250"/>
+    <ext cx="1143000" cy="771525"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -731,6 +753,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -739,13 +764,13 @@
     <from>
       <col>2</col>
       <colOff>66675</colOff>
-      <row>20</row>
+      <row>22</row>
       <rowOff>38100</rowOff>
     </from>
     <ext cx="1143000" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -756,6 +781,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -763,14 +791,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>76200</colOff>
-      <row>22</row>
+      <colOff>66675</colOff>
+      <row>23</row>
       <rowOff>38100</rowOff>
     </from>
-    <ext cx="1114425" cy="857250"/>
+    <ext cx="1143000" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -781,6 +809,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -788,14 +819,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>314325</colOff>
-      <row>23</row>
+      <colOff>133350</colOff>
+      <row>24</row>
       <rowOff>38100</rowOff>
     </from>
-    <ext cx="647700" cy="857250"/>
+    <ext cx="1000125" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -806,6 +837,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -814,13 +848,13 @@
     <from>
       <col>2</col>
       <colOff>66675</colOff>
-      <row>24</row>
-      <rowOff>76200</rowOff>
+      <row>25</row>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="1143000" cy="771525"/>
+    <ext cx="1143000" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -831,6 +865,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -840,12 +877,12 @@
       <col>2</col>
       <colOff>66675</colOff>
       <row>26</row>
-      <rowOff>38100</rowOff>
+      <rowOff>85725</rowOff>
     </from>
-    <ext cx="1143000" cy="857250"/>
+    <ext cx="1143000" cy="762000"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -856,6 +893,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -863,14 +903,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>66675</colOff>
+      <colOff>133350</colOff>
       <row>27</row>
       <rowOff>38100</rowOff>
     </from>
-    <ext cx="1143000" cy="857250"/>
+    <ext cx="1000125" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -881,6 +921,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -895,7 +938,7 @@
     <ext cx="1000125" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -906,6 +949,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -913,14 +959,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>66675</colOff>
+      <colOff>133350</colOff>
       <row>29</row>
       <rowOff>38100</rowOff>
     </from>
-    <ext cx="1143000" cy="857250"/>
+    <ext cx="1000125" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -931,6 +977,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -938,14 +987,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>66675</colOff>
+      <colOff>209550</colOff>
       <row>30</row>
-      <rowOff>85725</rowOff>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="1143000" cy="762000"/>
+    <ext cx="857250" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -956,6 +1005,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -963,14 +1015,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>133350</colOff>
+      <colOff>66675</colOff>
       <row>31</row>
       <rowOff>38100</rowOff>
     </from>
-    <ext cx="1000125" cy="857250"/>
+    <ext cx="1143000" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -981,6 +1033,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -988,14 +1043,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>133350</colOff>
+      <colOff>95250</colOff>
       <row>32</row>
       <rowOff>38100</rowOff>
     </from>
-    <ext cx="1000125" cy="857250"/>
+    <ext cx="1085850" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -1006,6 +1061,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1013,14 +1071,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>133350</colOff>
+      <colOff>371475</colOff>
       <row>33</row>
       <rowOff>38100</rowOff>
     </from>
-    <ext cx="1000125" cy="857250"/>
+    <ext cx="533400" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -1031,6 +1089,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1038,14 +1099,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>209550</colOff>
+      <colOff>104775</colOff>
       <row>34</row>
       <rowOff>38100</rowOff>
     </from>
-    <ext cx="857250" cy="857250"/>
+    <ext cx="1066800" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -1056,6 +1117,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1064,13 +1128,13 @@
     <from>
       <col>2</col>
       <colOff>66675</colOff>
-      <row>35</row>
-      <rowOff>38100</rowOff>
+      <row>36</row>
+      <rowOff>142875</rowOff>
     </from>
-    <ext cx="1143000" cy="857250"/>
+    <ext cx="1143000" cy="647700"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -1081,6 +1145,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1088,14 +1155,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>95250</colOff>
-      <row>36</row>
-      <rowOff>38100</rowOff>
+      <colOff>66675</colOff>
+      <row>37</row>
+      <rowOff>142875</rowOff>
     </from>
-    <ext cx="1085850" cy="857250"/>
+    <ext cx="1143000" cy="647700"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -1106,6 +1173,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1113,14 +1183,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>371475</colOff>
-      <row>37</row>
-      <rowOff>38100</rowOff>
+      <colOff>66675</colOff>
+      <row>38</row>
+      <rowOff>142875</rowOff>
     </from>
-    <ext cx="533400" cy="857250"/>
+    <ext cx="1143000" cy="647700"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -1131,6 +1201,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1138,14 +1211,14 @@
   <oneCellAnchor>
     <from>
       <col>2</col>
-      <colOff>104775</colOff>
-      <row>38</row>
-      <rowOff>38100</rowOff>
+      <colOff>66675</colOff>
+      <row>39</row>
+      <rowOff>142875</rowOff>
     </from>
-    <ext cx="1066800" cy="857250"/>
+    <ext cx="1143000" cy="647700"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -1156,6 +1229,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1164,13 +1240,13 @@
     <from>
       <col>2</col>
       <colOff>66675</colOff>
-      <row>40</row>
-      <rowOff>142875</rowOff>
+      <row>41</row>
+      <rowOff>104775</rowOff>
     </from>
-    <ext cx="1143000" cy="647700"/>
+    <ext cx="1143000" cy="714375"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -1181,6 +1257,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1189,13 +1268,13 @@
     <from>
       <col>2</col>
       <colOff>66675</colOff>
-      <row>41</row>
-      <rowOff>142875</rowOff>
+      <row>46</row>
+      <rowOff>38100</rowOff>
     </from>
-    <ext cx="1143000" cy="647700"/>
+    <ext cx="1143000" cy="857250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
@@ -1206,106 +1285,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>66675</colOff>
-      <row>42</row>
-      <rowOff>142875</rowOff>
-    </from>
-    <ext cx="1143000" cy="647700"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="30" name="Image 30" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>66675</colOff>
-      <row>43</row>
-      <rowOff>142875</rowOff>
-    </from>
-    <ext cx="1143000" cy="647700"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="31" name="Image 31" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>66675</colOff>
-      <row>45</row>
-      <rowOff>104775</rowOff>
-    </from>
-    <ext cx="1143000" cy="714375"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="32" name="Image 32" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId32"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>66675</colOff>
-      <row>50</row>
-      <rowOff>38100</rowOff>
-    </from>
-    <ext cx="1143000" cy="857250"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="33" name="Image 33" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId33"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1602,7 +1584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R72"/>
+  <dimension ref="A1:R68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1635,7 +1617,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Everything needed to build the robots with the arm, as of 2026-10-11. Prices are estimates in USD. Blue text = input you can change; yellow = fill in when you buy; green = from the Printed parts sheet.</t>
+          <t>Everything needed to build the robots with the arm, as of 2026-10-12. Prices are estimates in USD. Blue text = input you can change; yellow = fill in when you buy; green = from the Printed parts sheet.</t>
         </is>
       </c>
     </row>
@@ -2085,17 +2067,17 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Micro servo, metal gear (shoulder)</t>
+          <t>Micro servo, metal gear (MG90S)</t>
         </is>
       </c>
       <c r="C14" s="33" t="n"/>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>MG90S, with horns and screws</t>
+          <t>MG90S, with horns and screws: one for the shoulder, one for the gripper</t>
         </is>
       </c>
       <c r="E14" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
@@ -2107,7 +2089,7 @@
         <v/>
       </c>
       <c r="H14" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I14" s="35">
         <f>G14+H14</f>
@@ -2145,102 +2127,102 @@
       </c>
       <c r="R14" s="10" t="inlineStr">
         <is>
-          <t>Clone quality varies: buy from a well-reviewed store and test on arrival. Plugs straight into SERVO 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="74" customHeight="1">
-      <c r="A15" s="9" t="n">
+          <t>Both arm joints use the same servo (one part type to stock; metal gears survive a stalled gripper). SERVO 1 = shoulder, SERVO 2 = gripper. Clone quality varies: buy from a well-reviewed store and test on arrival. Each servo's bag has its horns and the tab screws that hold it in the arm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Battery and power</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="8" t="n"/>
+      <c r="H15" s="8" t="n"/>
+      <c r="I15" s="8" t="n"/>
+      <c r="J15" s="8" t="n"/>
+      <c r="K15" s="8" t="n"/>
+      <c r="L15" s="8" t="n"/>
+      <c r="M15" s="8" t="n"/>
+      <c r="N15" s="8" t="n"/>
+      <c r="O15" s="8" t="n"/>
+      <c r="P15" s="8" t="n"/>
+      <c r="Q15" s="8" t="n"/>
+      <c r="R15" s="8" t="n"/>
+    </row>
+    <row r="16" ht="74" customHeight="1">
+      <c r="A16" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Micro servo (gripper)</t>
-        </is>
-      </c>
-      <c r="C15" s="33" t="n"/>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>SG90, with horns and screws</t>
-        </is>
-      </c>
-      <c r="E15" s="34" t="n">
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>18650 Li-ion cell</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="n"/>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Branded (Samsung, LG, Molicel, EVE…), about 3000 mAh, 65 mm long, all the same type</t>
+        </is>
+      </c>
+      <c r="E16" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="G16" s="35">
+        <f>E16*$D$4</f>
+        <v/>
+      </c>
+      <c r="H16" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="35">
+        <f>G16+H16</f>
+        <v/>
+      </c>
+      <c r="J16" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="G15" s="35">
-        <f>E15*$D$4</f>
-        <v/>
-      </c>
-      <c r="H15" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" s="35">
-        <f>G15+H15</f>
-        <v/>
-      </c>
-      <c r="J15" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" s="35">
-        <f>IF(I15=0,0,ROUNDUP(I15/J15,0))</f>
-        <v/>
-      </c>
-      <c r="L15" s="36" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="M15" s="37">
-        <f>IF(Q15="Have already",0,K15*L15)</f>
-        <v/>
-      </c>
-      <c r="N15" s="10" t="inlineStr">
-        <is>
-          <t>AliExpress</t>
-        </is>
-      </c>
-      <c r="O15" s="15" t="inlineStr">
-        <is>
-          <t>Import</t>
-        </is>
-      </c>
-      <c r="P15" s="38" t="n"/>
-      <c r="Q15" s="15" t="inlineStr">
+      <c r="K16" s="35">
+        <f>IF(I16=0,0,ROUNDUP(I16/J16,0))</f>
+        <v/>
+      </c>
+      <c r="L16" s="36" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M16" s="37">
+        <f>IF(Q16="Have already",0,K16*L16)</f>
+        <v/>
+      </c>
+      <c r="N16" s="10" t="inlineStr">
+        <is>
+          <t>Local / South Africa</t>
+        </is>
+      </c>
+      <c r="O16" s="15" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="P16" s="38" t="n"/>
+      <c r="Q16" s="15" t="inlineStr">
         <is>
           <t>To buy</t>
         </is>
       </c>
-      <c r="R15" s="10" t="inlineStr">
-        <is>
-          <t>Plugs into SERVO 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Battery and power</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="8" t="n"/>
-      <c r="G16" s="8" t="n"/>
-      <c r="H16" s="8" t="n"/>
-      <c r="I16" s="8" t="n"/>
-      <c r="J16" s="8" t="n"/>
-      <c r="K16" s="8" t="n"/>
-      <c r="L16" s="8" t="n"/>
-      <c r="M16" s="8" t="n"/>
-      <c r="N16" s="8" t="n"/>
-      <c r="O16" s="8" t="n"/>
-      <c r="P16" s="8" t="n"/>
-      <c r="Q16" s="8" t="n"/>
-      <c r="R16" s="8" t="n"/>
+      <c r="R16" s="10" t="inlineStr">
+        <is>
+          <t>Don't ship from China: couriers refuse loose cells and fakes are common. Match the cells (same type, same voltage) before fitting. Protected cells are ~70 mm long and may not fit the holder.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="74" customHeight="1">
       <c r="A17" s="9" t="n">
@@ -2248,17 +2230,17 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>18650 Li-ion cell</t>
+          <t>3 × 18650 battery holder, parallel</t>
         </is>
       </c>
       <c r="C17" s="33" t="n"/>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>Branded (Samsung, LG, Molicel, EVE…), about 3000 mAh, 65 mm long, all the same type</t>
+          <t>61.6 × 78.4 mm, like the BatteryHolder3S in the model</t>
         </is>
       </c>
       <c r="E17" s="34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
@@ -2284,7 +2266,7 @@
         <v/>
       </c>
       <c r="L17" s="36" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="M17" s="37">
         <f>IF(Q17="Have already",0,K17*L17)</f>
@@ -2292,12 +2274,12 @@
       </c>
       <c r="N17" s="10" t="inlineStr">
         <is>
-          <t>Local / South Africa</t>
+          <t>AliExpress</t>
         </is>
       </c>
       <c r="O17" s="15" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Import</t>
         </is>
       </c>
       <c r="P17" s="38" t="n"/>
@@ -2308,7 +2290,7 @@
       </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
-          <t>Don't ship from China: couriers refuse loose cells and fakes are common. Match the cells (same type, same voltage) before fitting. Protected cells are ~70 mm long and may not fit the holder.</t>
+          <t>Wire it 1S3P (all cells in parallel). A holder sold as '3S' is wired in series and must be rewired: the board takes 4.2 V maximum. The chassis V-rails are sized for 61.6 × 78.4 mm.</t>
         </is>
       </c>
     </row>
@@ -2318,13 +2300,13 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>3 × 18650 battery holder, parallel</t>
+          <t>XT30 battery lead, female</t>
         </is>
       </c>
       <c r="C18" s="33" t="n"/>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>61.6 × 78.4 mm, like the BatteryHolder3S in the model</t>
+          <t>AMASS XT30U-F with 10–15 cm of 16 AWG silicone wire</t>
         </is>
       </c>
       <c r="E18" s="34" t="n">
@@ -2340,21 +2322,21 @@
         <v/>
       </c>
       <c r="H18" s="34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18" s="35">
         <f>G18+H18</f>
         <v/>
       </c>
       <c r="J18" s="34" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K18" s="35">
         <f>IF(I18=0,0,ROUNDUP(I18/J18,0))</f>
         <v/>
       </c>
       <c r="L18" s="36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M18" s="37">
         <f>IF(Q18="Have already",0,K18*L18)</f>
@@ -2362,7 +2344,7 @@
       </c>
       <c r="N18" s="10" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>AliExpress (AMASS store)</t>
         </is>
       </c>
       <c r="O18" s="15" t="inlineStr">
@@ -2378,97 +2360,50 @@
       </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
-          <t>Wire it 1S3P (all cells in parallel). A holder sold as '3S' is wired in series and must be rewired: the board takes 4.2 V maximum. The chassis V-rails are sized for 61.6 × 78.4 mm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="74" customHeight="1">
-      <c r="A19" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>1S Li-ion protection board (BMS)</t>
-        </is>
-      </c>
-      <c r="C19" s="33" t="n"/>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>Search: '1S 3.7V 18650 protection board 5A' (DW01 type)</t>
-        </is>
-      </c>
-      <c r="E19" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="G19" s="35">
-        <f>E19*$D$4</f>
-        <v/>
-      </c>
-      <c r="H19" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" s="35">
-        <f>G19+H19</f>
-        <v/>
-      </c>
-      <c r="J19" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="K19" s="35">
-        <f>IF(I19=0,0,ROUNDUP(I19/J19,0))</f>
-        <v/>
-      </c>
-      <c r="L19" s="36" t="n">
-        <v>2</v>
-      </c>
-      <c r="M19" s="37">
-        <f>IF(Q19="Have already",0,K19*L19)</f>
-        <v/>
-      </c>
-      <c r="N19" s="10" t="inlineStr">
-        <is>
-          <t>AliExpress</t>
-        </is>
-      </c>
-      <c r="O19" s="15" t="inlineStr">
-        <is>
-          <t>Import</t>
-        </is>
-      </c>
-      <c r="P19" s="38" t="n"/>
-      <c r="Q19" s="15" t="inlineStr">
-        <is>
-          <t>To buy</t>
-        </is>
-      </c>
-      <c r="R19" s="10" t="inlineStr">
-        <is>
-          <t>Recommended: the controller has no low-battery cut-off, so this stops the cells being over-drained. Goes between the holder and the XT30 lead. Pick one rated 5 A or more.</t>
-        </is>
-      </c>
+          <t>The board has the male XT30 (XT30UPB-M), so the battery side needs the female plug. Solder it straight to the holder's leads and insulate the joints (heat-shrink or tape you already have).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Cables</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="8" t="n"/>
+      <c r="H19" s="8" t="n"/>
+      <c r="I19" s="8" t="n"/>
+      <c r="J19" s="8" t="n"/>
+      <c r="K19" s="8" t="n"/>
+      <c r="L19" s="8" t="n"/>
+      <c r="M19" s="8" t="n"/>
+      <c r="N19" s="8" t="n"/>
+      <c r="O19" s="8" t="n"/>
+      <c r="P19" s="8" t="n"/>
+      <c r="Q19" s="8" t="n"/>
+      <c r="R19" s="8" t="n"/>
     </row>
     <row r="20" ht="74" customHeight="1">
       <c r="A20" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>XT30 battery lead, female</t>
+          <t>Dupont jumper wires, female-female, 20 cm</t>
         </is>
       </c>
       <c r="C20" s="33" t="n"/>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>AMASS XT30U-F with 10–15 cm of 16 AWG silicone wire</t>
+          <t>4 for the ultrasonic (J403) + 5 for the line sensor (J404)</t>
         </is>
       </c>
       <c r="E20" s="34" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
@@ -2480,21 +2415,21 @@
         <v/>
       </c>
       <c r="H20" s="34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20" s="35">
         <f>G20+H20</f>
         <v/>
       </c>
       <c r="J20" s="34" t="n">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="K20" s="35">
         <f>IF(I20=0,0,ROUNDUP(I20/J20,0))</f>
         <v/>
       </c>
       <c r="L20" s="36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M20" s="37">
         <f>IF(Q20="Have already",0,K20*L20)</f>
@@ -2502,7 +2437,7 @@
       </c>
       <c r="N20" s="10" t="inlineStr">
         <is>
-          <t>AliExpress (AMASS store)</t>
+          <t>AliExpress</t>
         </is>
       </c>
       <c r="O20" s="15" t="inlineStr">
@@ -2518,23 +2453,23 @@
       </c>
       <c r="R20" s="10" t="inlineStr">
         <is>
-          <t>The board has the male XT30 (XT30UPB-M), so the battery side needs the female plug.</t>
+          <t>Usually sold as a 40-wire strip.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="74" customHeight="1">
       <c r="A21" s="9" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Heat-shrink tubing assortment</t>
+          <t>USB charger, 5 V 2 A (optional)</t>
         </is>
       </c>
       <c r="C21" s="33" t="n"/>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>For the battery wiring joints</t>
+          <t>Any phone charger with a USB-C or USB-A port</t>
         </is>
       </c>
       <c r="E21" s="34" t="n">
@@ -2542,7 +2477,7 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G21" s="35">
@@ -2550,7 +2485,7 @@
         <v/>
       </c>
       <c r="H21" s="34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21" s="35">
         <f>G21+H21</f>
@@ -2564,7 +2499,7 @@
         <v/>
       </c>
       <c r="L21" s="36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M21" s="37">
         <f>IF(Q21="Have already",0,K21*L21)</f>
@@ -2572,12 +2507,12 @@
       </c>
       <c r="N21" s="10" t="inlineStr">
         <is>
-          <t>AliExpress / local</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="O21" s="15" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="P21" s="38" t="n"/>
@@ -2588,14 +2523,14 @@
       </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
-          <t>One-off. Skip if you have some.</t>
+          <t>Set 'Per robot' to 1 if the users don't have one. The board draws up to 1.65 A from USB.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Cables</t>
+          <t>Screws, inserts and small hardware (with the arm and one bus clip)</t>
         </is>
       </c>
       <c r="B22" s="8" t="n"/>
@@ -2617,21 +2552,21 @@
     </row>
     <row r="23" ht="74" customHeight="1">
       <c r="A23" s="9" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Dupont jumper wires, female-female, 20 cm</t>
+          <t>M2 heat-set insert</t>
         </is>
       </c>
       <c r="C23" s="33" t="n"/>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>4 for the ultrasonic (J403) + 5 for the line sensor (J404)</t>
+          <t>For Ø3.2 mm holes (e.g. M2 × 3 × 3.2 OD)</t>
         </is>
       </c>
       <c r="E23" s="34" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
@@ -2643,14 +2578,14 @@
         <v/>
       </c>
       <c r="H23" s="34" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I23" s="35">
         <f>G23+H23</f>
         <v/>
       </c>
       <c r="J23" s="34" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="K23" s="35">
         <f>IF(I23=0,0,ROUNDUP(I23/J23,0))</f>
@@ -2681,27 +2616,27 @@
       </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
-          <t>Usually sold as a 40-wire strip.</t>
+          <t>4: melted into the 4 bosses under the controller's corner holes; the board screws into them.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="74" customHeight="1">
       <c r="A24" s="9" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>USB-C cable (data)</t>
+          <t>M3 heat-set insert, short</t>
         </is>
       </c>
       <c r="C24" s="33" t="n"/>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>USB-A or USB-C to USB-C; must carry data</t>
+          <t>For Ø4.0 mm holes (e.g. M3 × 4 × 4.0 OD)</t>
         </is>
       </c>
       <c r="E24" s="34" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2713,21 +2648,21 @@
         <v/>
       </c>
       <c r="H24" s="34" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I24" s="35">
         <f>G24+H24</f>
         <v/>
       </c>
       <c r="J24" s="34" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K24" s="35">
         <f>IF(I24=0,0,ROUNDUP(I24/J24,0))</f>
         <v/>
       </c>
       <c r="L24" s="36" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="M24" s="37">
         <f>IF(Q24="Have already",0,K24*L24)</f>
@@ -2735,7 +2670,7 @@
       </c>
       <c r="N24" s="10" t="inlineStr">
         <is>
-          <t>AliExpress / local</t>
+          <t>AliExpress</t>
         </is>
       </c>
       <c r="O24" s="15" t="inlineStr">
@@ -2751,27 +2686,27 @@
       </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
-          <t>For programming and charging. Charge-only cables won't program the board.</t>
+          <t>6: 2 in the dock tower tops (arm base + sonar bracket), 1 in each ballast clip (2), 1 in the bus clip's tab, 1 in the bus clip's accessory boss.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="74" customHeight="1">
       <c r="A25" s="9" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>USB charger, 5 V 2 A (optional)</t>
+          <t>M2 × 6 pan head machine screw</t>
         </is>
       </c>
       <c r="C25" s="33" t="n"/>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>Any phone charger with a USB-C or USB-A port</t>
+          <t>Into the M2 inserts</t>
         </is>
       </c>
       <c r="E25" s="34" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
@@ -2783,21 +2718,21 @@
         <v/>
       </c>
       <c r="H25" s="34" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I25" s="35">
         <f>G25+H25</f>
         <v/>
       </c>
       <c r="J25" s="34" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="K25" s="35">
         <f>IF(I25=0,0,ROUNDUP(I25/J25,0))</f>
         <v/>
       </c>
       <c r="L25" s="36" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="M25" s="37">
         <f>IF(Q25="Have already",0,K25*L25)</f>
@@ -2805,12 +2740,12 @@
       </c>
       <c r="N25" s="10" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>AliExpress</t>
         </is>
       </c>
       <c r="O25" s="15" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Import</t>
         </is>
       </c>
       <c r="P25" s="38" t="n"/>
@@ -2821,32 +2756,79 @@
       </c>
       <c r="R25" s="10" t="inlineStr">
         <is>
-          <t>Set 'Per robot' to 1 if the users don't have one. The board draws up to 1.65 A from USB.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Screws, inserts and small hardware (with the arm and one bus clip)</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="n"/>
-      <c r="D26" s="8" t="n"/>
-      <c r="E26" s="8" t="n"/>
-      <c r="F26" s="8" t="n"/>
-      <c r="G26" s="8" t="n"/>
-      <c r="H26" s="8" t="n"/>
-      <c r="I26" s="8" t="n"/>
-      <c r="J26" s="8" t="n"/>
-      <c r="K26" s="8" t="n"/>
-      <c r="L26" s="8" t="n"/>
-      <c r="M26" s="8" t="n"/>
-      <c r="N26" s="8" t="n"/>
-      <c r="O26" s="8" t="n"/>
-      <c r="P26" s="8" t="n"/>
-      <c r="Q26" s="8" t="n"/>
-      <c r="R26" s="8" t="n"/>
+          <t>4: controller onto the deck, into the M2 inserts. Tip: one M2/M3 screw assortment kit covers most of this section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="74" customHeight="1">
+      <c r="A26" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>M2 × 6 pan head self-tapping screw</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="n"/>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>Wheel onto the motor shaft</t>
+        </is>
+      </c>
+      <c r="E26" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="G26" s="35">
+        <f>E26*$D$4</f>
+        <v/>
+      </c>
+      <c r="H26" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" s="35">
+        <f>G26+H26</f>
+        <v/>
+      </c>
+      <c r="J26" s="34" t="n">
+        <v>50</v>
+      </c>
+      <c r="K26" s="35">
+        <f>IF(I26=0,0,ROUNDUP(I26/J26,0))</f>
+        <v/>
+      </c>
+      <c r="L26" s="36" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M26" s="37">
+        <f>IF(Q26="Have already",0,K26*L26)</f>
+        <v/>
+      </c>
+      <c r="N26" s="10" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="O26" s="15" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="P26" s="38" t="n"/>
+      <c r="Q26" s="15" t="inlineStr">
+        <is>
+          <t>To buy</t>
+        </is>
+      </c>
+      <c r="R26" s="10" t="inlineStr">
+        <is>
+          <t>2: one per wheel, into the motor shaft's centre hole, with a washer under the head.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="74" customHeight="1">
       <c r="A27" s="9" t="n">
@@ -2854,17 +2836,13 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>M2 heat-set insert</t>
+          <t>M2 flat washer</t>
         </is>
       </c>
       <c r="C27" s="33" t="n"/>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>For Ø3.2 mm holes (e.g. M2 × 3 × 3.2 OD)</t>
-        </is>
-      </c>
+      <c r="D27" s="10" t="inlineStr"/>
       <c r="E27" s="34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2876,7 +2854,7 @@
         <v/>
       </c>
       <c r="H27" s="34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I27" s="35">
         <f>G27+H27</f>
@@ -2890,7 +2868,7 @@
         <v/>
       </c>
       <c r="L27" s="36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M27" s="37">
         <f>IF(Q27="Have already",0,K27*L27)</f>
@@ -2914,7 +2892,7 @@
       </c>
       <c r="R27" s="10" t="inlineStr">
         <is>
-          <t>Board onto the deck.</t>
+          <t>2: one under each wheel screw.</t>
         </is>
       </c>
     </row>
@@ -2924,17 +2902,13 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>M3 heat-set insert, short</t>
+          <t>M2 × 8 pan head screw</t>
         </is>
       </c>
       <c r="C28" s="33" t="n"/>
-      <c r="D28" s="10" t="inlineStr">
-        <is>
-          <t>For Ø4.0 mm holes (e.g. M3 × 4 × 4.0 OD)</t>
-        </is>
-      </c>
+      <c r="D28" s="10" t="inlineStr"/>
       <c r="E28" s="34" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
@@ -2946,21 +2920,21 @@
         <v/>
       </c>
       <c r="H28" s="34" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I28" s="35">
         <f>G28+H28</f>
         <v/>
       </c>
       <c r="J28" s="34" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K28" s="35">
         <f>IF(I28=0,0,ROUNDUP(I28/J28,0))</f>
         <v/>
       </c>
       <c r="L28" s="36" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="M28" s="37">
         <f>IF(Q28="Have already",0,K28*L28)</f>
@@ -2984,7 +2958,7 @@
       </c>
       <c r="R28" s="10" t="inlineStr">
         <is>
-          <t>2 dock towers, 3 clips (bus + 2 ballast), 1 bus-clip accessory boss.</t>
+          <t>1: shoulder servo horn centre screw, through the boom plate (the servo's own screw is too short).</t>
         </is>
       </c>
     </row>
@@ -2994,17 +2968,13 @@
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>M2 × 6 pan head machine screw</t>
+          <t>M2 × 5 pan head screw</t>
         </is>
       </c>
       <c r="C29" s="33" t="n"/>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>Into the M2 inserts</t>
-        </is>
-      </c>
+      <c r="D29" s="10" t="inlineStr"/>
       <c r="E29" s="34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
@@ -3016,7 +2986,7 @@
         <v/>
       </c>
       <c r="H29" s="34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I29" s="35">
         <f>G29+H29</f>
@@ -3054,7 +3024,7 @@
       </c>
       <c r="R29" s="10" t="inlineStr">
         <is>
-          <t>Board onto the deck. Tip: one M2/M3 screw assortment kit covers most of this section.</t>
+          <t>2: shoulder horn arm to the right boom plate.</t>
         </is>
       </c>
     </row>
@@ -3064,17 +3034,13 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>M2 × 6 pan head self-tapping screw</t>
+          <t>M2 × 4 pan head screw</t>
         </is>
       </c>
       <c r="C30" s="33" t="n"/>
-      <c r="D30" s="10" t="inlineStr">
-        <is>
-          <t>Wheel onto the motor shaft</t>
-        </is>
-      </c>
+      <c r="D30" s="10" t="inlineStr"/>
       <c r="E30" s="34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
@@ -3124,7 +3090,7 @@
       </c>
       <c r="R30" s="10" t="inlineStr">
         <is>
-          <t>Into the shaft's centre hole, with a washer.</t>
+          <t>3: gripper horn: centre screw into the servo + 2 through the horn arm into the driven jaw.</t>
         </is>
       </c>
     </row>
@@ -3134,7 +3100,7 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>M2 flat washer</t>
+          <t>M3 × 10 socket head screw</t>
         </is>
       </c>
       <c r="C31" s="33" t="n"/>
@@ -3159,14 +3125,14 @@
         <v/>
       </c>
       <c r="J31" s="34" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K31" s="35">
         <f>IF(I31=0,0,ROUNDUP(I31/J31,0))</f>
         <v/>
       </c>
       <c r="L31" s="36" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="M31" s="37">
         <f>IF(Q31="Have already",0,K31*L31)</f>
@@ -3190,7 +3156,7 @@
       </c>
       <c r="R31" s="10" t="inlineStr">
         <is>
-          <t>Under the wheel screws.</t>
+          <t>2: through the arm base and sonar bracket into the dock-tower inserts (M3 × 8 if you build without the arm).</t>
         </is>
       </c>
     </row>
@@ -3200,7 +3166,7 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>M2 × 8 pan head screw</t>
+          <t>M3 × 8 pan head self-tapping screw</t>
         </is>
       </c>
       <c r="C32" s="33" t="n"/>
@@ -3256,7 +3222,7 @@
       </c>
       <c r="R32" s="10" t="inlineStr">
         <is>
-          <t>Shoulder horn centre screw (the servo's own screw is too short).</t>
+          <t>1: pivot of the idle (right) jaw; self-taps into the arm.</t>
         </is>
       </c>
     </row>
@@ -3266,13 +3232,13 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>M2 × 5 pan head screw</t>
+          <t>M3 × 8 thumb screw (knurled head)</t>
         </is>
       </c>
       <c r="C33" s="33" t="n"/>
       <c r="D33" s="10" t="inlineStr"/>
       <c r="E33" s="34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -3284,21 +3250,21 @@
         <v/>
       </c>
       <c r="H33" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I33" s="35">
         <f>G33+H33</f>
         <v/>
       </c>
       <c r="J33" s="34" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="K33" s="35">
         <f>IF(I33=0,0,ROUNDUP(I33/J33,0))</f>
         <v/>
       </c>
       <c r="L33" s="36" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="M33" s="37">
         <f>IF(Q33="Have already",0,K33*L33)</f>
@@ -3322,7 +3288,7 @@
       </c>
       <c r="R33" s="10" t="inlineStr">
         <is>
-          <t>Shoulder horn arm to the boom plate.</t>
+          <t>3: one each on the bus clip and the 2 ballast clips; it presses on the deck and locks the clip.</t>
         </is>
       </c>
     </row>
@@ -3332,13 +3298,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>M2 × 4 pan head screw</t>
+          <t>M8 hex nut</t>
         </is>
       </c>
       <c r="C34" s="33" t="n"/>
-      <c r="D34" s="10" t="inlineStr"/>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>Plain steel, about 5 g each</t>
+        </is>
+      </c>
       <c r="E34" s="34" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -3350,21 +3320,21 @@
         <v/>
       </c>
       <c r="H34" s="34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I34" s="35">
         <f>G34+H34</f>
         <v/>
       </c>
       <c r="J34" s="34" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="K34" s="35">
         <f>IF(I34=0,0,ROUNDUP(I34/J34,0))</f>
         <v/>
       </c>
       <c r="L34" s="36" t="n">
-        <v>1.5</v>
+        <v>0.1</v>
       </c>
       <c r="M34" s="37">
         <f>IF(Q34="Have already",0,K34*L34)</f>
@@ -3372,12 +3342,12 @@
       </c>
       <c r="N34" s="10" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>Local hardware shop</t>
         </is>
       </c>
       <c r="O34" s="15" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="P34" s="38" t="n"/>
@@ -3388,7 +3358,7 @@
       </c>
       <c r="R34" s="10" t="inlineStr">
         <is>
-          <t>Gripper horn: centre screw + 2 into the jaw.</t>
+          <t>6: 3 in each ballast clip on the rear wall. Needed when the arm is fitted.</t>
         </is>
       </c>
     </row>
@@ -3398,11 +3368,15 @@
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>M3 × 10 socket head screw</t>
+          <t>½" (12.7 mm) steel ball</t>
         </is>
       </c>
       <c r="C35" s="33" t="n"/>
-      <c r="D35" s="10" t="inlineStr"/>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>Bearing balls or slingshot ammo; 12.7 mm glass marbles also work</t>
+        </is>
+      </c>
       <c r="E35" s="34" t="n">
         <v>2</v>
       </c>
@@ -3423,14 +3397,14 @@
         <v/>
       </c>
       <c r="J35" s="34" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="K35" s="35">
         <f>IF(I35=0,0,ROUNDUP(I35/J35,0))</f>
         <v/>
       </c>
       <c r="L35" s="36" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="M35" s="37">
         <f>IF(Q35="Have already",0,K35*L35)</f>
@@ -3438,7 +3412,7 @@
       </c>
       <c r="N35" s="10" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>AliExpress / local bearing shop</t>
         </is>
       </c>
       <c r="O35" s="15" t="inlineStr">
@@ -3454,115 +3428,78 @@
       </c>
       <c r="R35" s="10" t="inlineStr">
         <is>
-          <t>Sonar bracket + arm base into the dock (M3 × 8 if no arm).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="74" customHeight="1">
-      <c r="A36" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>M3 × 8 pan head self-tapping screw</t>
-        </is>
-      </c>
-      <c r="C36" s="33" t="n"/>
-      <c r="D36" s="10" t="inlineStr"/>
-      <c r="E36" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="G36" s="35">
-        <f>E36*$D$4</f>
-        <v/>
-      </c>
-      <c r="H36" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="I36" s="35">
-        <f>G36+H36</f>
-        <v/>
-      </c>
-      <c r="J36" s="34" t="n">
-        <v>50</v>
-      </c>
-      <c r="K36" s="35">
-        <f>IF(I36=0,0,ROUNDUP(I36/J36,0))</f>
-        <v/>
-      </c>
-      <c r="L36" s="36" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="M36" s="37">
-        <f>IF(Q36="Have already",0,K36*L36)</f>
-        <v/>
-      </c>
-      <c r="N36" s="10" t="inlineStr">
-        <is>
-          <t>AliExpress</t>
-        </is>
-      </c>
-      <c r="O36" s="15" t="inlineStr">
-        <is>
-          <t>Import</t>
-        </is>
-      </c>
-      <c r="P36" s="38" t="n"/>
-      <c r="Q36" s="15" t="inlineStr">
-        <is>
-          <t>To buy</t>
-        </is>
-      </c>
-      <c r="R36" s="10" t="inlineStr">
-        <is>
-          <t>Idle jaw pivot.</t>
-        </is>
-      </c>
+          <t>2: rear casters, press-fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>3D printing filament (grams, from the Printed parts sheet)</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="n"/>
+      <c r="D36" s="8" t="n"/>
+      <c r="E36" s="8" t="n"/>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="8" t="n"/>
+      <c r="H36" s="8" t="n"/>
+      <c r="I36" s="8" t="n"/>
+      <c r="J36" s="8" t="n"/>
+      <c r="K36" s="8" t="n"/>
+      <c r="L36" s="8" t="n"/>
+      <c r="M36" s="8" t="n"/>
+      <c r="N36" s="8" t="n"/>
+      <c r="O36" s="8" t="n"/>
+      <c r="P36" s="8" t="n"/>
+      <c r="Q36" s="8" t="n"/>
+      <c r="R36" s="8" t="n"/>
     </row>
     <row r="37" ht="74" customHeight="1">
       <c r="A37" s="9" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>M3 × 8 thumb screw (knurled head)</t>
+          <t>PETG filament, yellow</t>
         </is>
       </c>
       <c r="C37" s="33" t="n"/>
-      <c r="D37" s="10" t="inlineStr"/>
-      <c r="E37" s="34" t="n">
-        <v>3</v>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>1 kg spool</t>
+        </is>
+      </c>
+      <c r="E37" s="39">
+        <f>'Printed parts'!C24</f>
+        <v/>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>g</t>
         </is>
       </c>
       <c r="G37" s="35">
         <f>E37*$D$4</f>
         <v/>
       </c>
-      <c r="H37" s="34" t="n">
-        <v>1</v>
+      <c r="H37" s="39">
+        <f>'Printed parts'!D24</f>
+        <v/>
       </c>
       <c r="I37" s="35">
         <f>G37+H37</f>
         <v/>
       </c>
       <c r="J37" s="34" t="n">
-        <v>20</v>
+        <v>1000</v>
       </c>
       <c r="K37" s="35">
         <f>IF(I37=0,0,ROUNDUP(I37/J37,0))</f>
         <v/>
       </c>
       <c r="L37" s="36" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="M37" s="37">
         <f>IF(Q37="Have already",0,K37*L37)</f>
@@ -3570,12 +3507,12 @@
       </c>
       <c r="N37" s="10" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>Local / Bambu store</t>
         </is>
       </c>
       <c r="O37" s="15" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="P37" s="38" t="n"/>
@@ -3586,53 +3523,55 @@
       </c>
       <c r="R37" s="10" t="inlineStr">
         <is>
-          <t>Bus clip + 2 ballast clips (presses on the deck).</t>
+          <t>Chassis, sonar pod, arm and arm base.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="74" customHeight="1">
       <c r="A38" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>M8 hex nut</t>
+          <t>PETG filament, black</t>
         </is>
       </c>
       <c r="C38" s="33" t="n"/>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>Plain steel, about 5 g each</t>
-        </is>
-      </c>
-      <c r="E38" s="34" t="n">
-        <v>6</v>
+          <t>1 kg spool</t>
+        </is>
+      </c>
+      <c r="E38" s="39">
+        <f>'Printed parts'!C25</f>
+        <v/>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>g</t>
         </is>
       </c>
       <c r="G38" s="35">
         <f>E38*$D$4</f>
         <v/>
       </c>
-      <c r="H38" s="34" t="n">
-        <v>0</v>
+      <c r="H38" s="39">
+        <f>'Printed parts'!D25</f>
+        <v/>
       </c>
       <c r="I38" s="35">
         <f>G38+H38</f>
         <v/>
       </c>
       <c r="J38" s="34" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="K38" s="35">
         <f>IF(I38=0,0,ROUNDUP(I38/J38,0))</f>
         <v/>
       </c>
       <c r="L38" s="36" t="n">
-        <v>0.1</v>
+        <v>20</v>
       </c>
       <c r="M38" s="37">
         <f>IF(Q38="Have already",0,K38*L38)</f>
@@ -3640,7 +3579,7 @@
       </c>
       <c r="N38" s="10" t="inlineStr">
         <is>
-          <t>Local hardware shop</t>
+          <t>Local / Bambu store</t>
         </is>
       </c>
       <c r="O38" s="15" t="inlineStr">
@@ -3656,53 +3595,55 @@
       </c>
       <c r="R38" s="10" t="inlineStr">
         <is>
-          <t>Ballast: 3 in each ballast clip. Needed when the arm is fitted.</t>
+          <t>Line sled, jaws, clips, test pieces. Mark 'Have already' if you have black.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="74" customHeight="1">
       <c r="A39" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>½" (12.7 mm) steel ball</t>
+          <t>PETG filament, dark teal</t>
         </is>
       </c>
       <c r="C39" s="33" t="n"/>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>Bearing balls or slingshot ammo; 12.7 mm glass marbles also work</t>
-        </is>
-      </c>
-      <c r="E39" s="34" t="n">
-        <v>2</v>
+          <t>1 kg spool</t>
+        </is>
+      </c>
+      <c r="E39" s="39">
+        <f>'Printed parts'!C26</f>
+        <v/>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>g</t>
         </is>
       </c>
       <c r="G39" s="35">
         <f>E39*$D$4</f>
         <v/>
       </c>
-      <c r="H39" s="34" t="n">
-        <v>2</v>
+      <c r="H39" s="39">
+        <f>'Printed parts'!D26</f>
+        <v/>
       </c>
       <c r="I39" s="35">
         <f>G39+H39</f>
         <v/>
       </c>
       <c r="J39" s="34" t="n">
-        <v>20</v>
+        <v>1000</v>
       </c>
       <c r="K39" s="35">
         <f>IF(I39=0,0,ROUNDUP(I39/J39,0))</f>
         <v/>
       </c>
       <c r="L39" s="36" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="M39" s="37">
         <f>IF(Q39="Have already",0,K39*L39)</f>
@@ -3710,12 +3651,12 @@
       </c>
       <c r="N39" s="10" t="inlineStr">
         <is>
-          <t>AliExpress / local bearing shop</t>
+          <t>Local / Bambu store</t>
         </is>
       </c>
       <c r="O39" s="15" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="P39" s="38" t="n"/>
@@ -3726,150 +3667,148 @@
       </c>
       <c r="R39" s="10" t="inlineStr">
         <is>
-          <t>Rear casters, press-fit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>3D printing filament (grams, from the Printed parts sheet)</t>
-        </is>
-      </c>
-      <c r="B40" s="8" t="n"/>
-      <c r="D40" s="8" t="n"/>
-      <c r="E40" s="8" t="n"/>
-      <c r="F40" s="8" t="n"/>
-      <c r="G40" s="8" t="n"/>
-      <c r="H40" s="8" t="n"/>
-      <c r="I40" s="8" t="n"/>
-      <c r="J40" s="8" t="n"/>
-      <c r="K40" s="8" t="n"/>
-      <c r="L40" s="8" t="n"/>
-      <c r="M40" s="8" t="n"/>
-      <c r="N40" s="8" t="n"/>
-      <c r="O40" s="8" t="n"/>
-      <c r="P40" s="8" t="n"/>
-      <c r="Q40" s="8" t="n"/>
-      <c r="R40" s="8" t="n"/>
-    </row>
-    <row r="41" ht="74" customHeight="1">
-      <c r="A41" s="9" t="n">
-        <v>28</v>
-      </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>PETG filament, yellow</t>
-        </is>
-      </c>
-      <c r="C41" s="33" t="n"/>
-      <c r="D41" s="10" t="inlineStr">
-        <is>
-          <t>1 kg spool</t>
-        </is>
-      </c>
-      <c r="E41" s="39">
-        <f>'Printed parts'!C24</f>
-        <v/>
-      </c>
-      <c r="F41" s="9" t="inlineStr">
+          <t>Wheels only. Print them black instead to skip this spool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="74" customHeight="1">
+      <c r="A40" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>TPU 95A filament, black</t>
+        </is>
+      </c>
+      <c r="C40" s="33" t="n"/>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>250–1000 g spool</t>
+        </is>
+      </c>
+      <c r="E40" s="39">
+        <f>'Printed parts'!C27</f>
+        <v/>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
         <is>
           <t>g</t>
         </is>
       </c>
-      <c r="G41" s="35">
-        <f>E41*$D$4</f>
-        <v/>
-      </c>
-      <c r="H41" s="39">
-        <f>'Printed parts'!D24</f>
-        <v/>
-      </c>
-      <c r="I41" s="35">
-        <f>G41+H41</f>
-        <v/>
-      </c>
-      <c r="J41" s="34" t="n">
+      <c r="G40" s="35">
+        <f>E40*$D$4</f>
+        <v/>
+      </c>
+      <c r="H40" s="39">
+        <f>'Printed parts'!D27</f>
+        <v/>
+      </c>
+      <c r="I40" s="35">
+        <f>G40+H40</f>
+        <v/>
+      </c>
+      <c r="J40" s="34" t="n">
         <v>1000</v>
       </c>
-      <c r="K41" s="35">
-        <f>IF(I41=0,0,ROUNDUP(I41/J41,0))</f>
-        <v/>
-      </c>
-      <c r="L41" s="36" t="n">
-        <v>20</v>
-      </c>
-      <c r="M41" s="37">
-        <f>IF(Q41="Have already",0,K41*L41)</f>
-        <v/>
-      </c>
-      <c r="N41" s="10" t="inlineStr">
+      <c r="K40" s="35">
+        <f>IF(I40=0,0,ROUNDUP(I40/J40,0))</f>
+        <v/>
+      </c>
+      <c r="L40" s="36" t="n">
+        <v>25</v>
+      </c>
+      <c r="M40" s="37">
+        <f>IF(Q40="Have already",0,K40*L40)</f>
+        <v/>
+      </c>
+      <c r="N40" s="10" t="inlineStr">
         <is>
           <t>Local / Bambu store</t>
         </is>
       </c>
-      <c r="O41" s="15" t="inlineStr">
+      <c r="O40" s="15" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="P41" s="38" t="n"/>
-      <c r="Q41" s="15" t="inlineStr">
+      <c r="P40" s="38" t="n"/>
+      <c r="Q40" s="15" t="inlineStr">
         <is>
           <t>To buy</t>
         </is>
       </c>
-      <c r="R41" s="10" t="inlineStr">
-        <is>
-          <t>Chassis, sonar pod, arm and arm base.</t>
-        </is>
-      </c>
+      <c r="R40" s="10" t="inlineStr">
+        <is>
+          <t>Tyres only; about 25 g needed, so a small spool is enough.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Packaging (optional)</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="n"/>
+      <c r="D41" s="8" t="n"/>
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="8" t="n"/>
+      <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
+      <c r="J41" s="8" t="n"/>
+      <c r="K41" s="8" t="n"/>
+      <c r="L41" s="8" t="n"/>
+      <c r="M41" s="8" t="n"/>
+      <c r="N41" s="8" t="n"/>
+      <c r="O41" s="8" t="n"/>
+      <c r="P41" s="8" t="n"/>
+      <c r="Q41" s="8" t="n"/>
+      <c r="R41" s="8" t="n"/>
     </row>
     <row r="42" ht="74" customHeight="1">
       <c r="A42" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>PETG filament, black</t>
+          <t>Mailer box + printed quick-start guide</t>
         </is>
       </c>
       <c r="C42" s="33" t="n"/>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>1 kg spool</t>
-        </is>
-      </c>
-      <c r="E42" s="39">
-        <f>'Printed parts'!C25</f>
-        <v/>
+          <t>Design in mech/robot/packaging (273 × 203 × 83 mm outer)</t>
+        </is>
+      </c>
+      <c r="E42" s="34" t="n">
+        <v>1</v>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G42" s="35">
         <f>E42*$D$4</f>
         <v/>
       </c>
-      <c r="H42" s="39">
-        <f>'Printed parts'!D25</f>
-        <v/>
+      <c r="H42" s="34" t="n">
+        <v>0</v>
       </c>
       <c r="I42" s="35">
         <f>G42+H42</f>
         <v/>
       </c>
       <c r="J42" s="34" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="K42" s="35">
         <f>IF(I42=0,0,ROUNDUP(I42/J42,0))</f>
         <v/>
       </c>
       <c r="L42" s="36" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="M42" s="37">
         <f>IF(Q42="Have already",0,K42*L42)</f>
@@ -3877,7 +3816,7 @@
       </c>
       <c r="N42" s="10" t="inlineStr">
         <is>
-          <t>Local / Bambu store</t>
+          <t>Local print shop</t>
         </is>
       </c>
       <c r="O42" s="15" t="inlineStr">
@@ -3893,127 +3832,80 @@
       </c>
       <c r="R42" s="10" t="inlineStr">
         <is>
-          <t>Line sled, jaws, clips, test pieces. Mark 'Have already' if you have black.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="74" customHeight="1">
-      <c r="A43" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t>PETG filament, dark teal</t>
-        </is>
-      </c>
-      <c r="C43" s="33" t="n"/>
-      <c r="D43" s="10" t="inlineStr">
-        <is>
-          <t>1 kg spool</t>
-        </is>
-      </c>
-      <c r="E43" s="39">
-        <f>'Printed parts'!C26</f>
-        <v/>
-      </c>
-      <c r="F43" s="9" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="G43" s="35">
-        <f>E43*$D$4</f>
-        <v/>
-      </c>
-      <c r="H43" s="39">
-        <f>'Printed parts'!D26</f>
-        <v/>
-      </c>
-      <c r="I43" s="35">
-        <f>G43+H43</f>
-        <v/>
-      </c>
-      <c r="J43" s="34" t="n">
-        <v>1000</v>
-      </c>
-      <c r="K43" s="35">
-        <f>IF(I43=0,0,ROUNDUP(I43/J43,0))</f>
-        <v/>
-      </c>
-      <c r="L43" s="36" t="n">
-        <v>20</v>
-      </c>
-      <c r="M43" s="37">
-        <f>IF(Q43="Have already",0,K43*L43)</f>
-        <v/>
-      </c>
-      <c r="N43" s="10" t="inlineStr">
-        <is>
-          <t>Local / Bambu store</t>
-        </is>
-      </c>
-      <c r="O43" s="15" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="P43" s="38" t="n"/>
-      <c r="Q43" s="15" t="inlineStr">
-        <is>
-          <t>To buy</t>
-        </is>
-      </c>
-      <c r="R43" s="10" t="inlineStr">
-        <is>
-          <t>Wheels only. Print them black instead to skip this spool.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="74" customHeight="1">
+          <t>Estimate from the costing model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>Shipping (estimates; replace with the checkout price)</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="n"/>
+      <c r="D43" s="8" t="n"/>
+      <c r="E43" s="8" t="n"/>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="8" t="n"/>
+      <c r="H43" s="8" t="n"/>
+      <c r="I43" s="8" t="n"/>
+      <c r="J43" s="8" t="n"/>
+      <c r="K43" s="8" t="n"/>
+      <c r="L43" s="8" t="n"/>
+      <c r="M43" s="8" t="n"/>
+      <c r="N43" s="8" t="n"/>
+      <c r="O43" s="8" t="n"/>
+      <c r="P43" s="8" t="n"/>
+      <c r="Q43" s="8" t="n"/>
+      <c r="R43" s="8" t="n"/>
+    </row>
+    <row r="44">
       <c r="A44" s="9" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>TPU 95A filament, black</t>
-        </is>
-      </c>
-      <c r="C44" s="33" t="n"/>
+          <t>Shipping: SparkFun order (motors)</t>
+        </is>
+      </c>
+      <c r="C44" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>250–1000 g spool</t>
-        </is>
-      </c>
-      <c r="E44" s="39">
-        <f>'Printed parts'!C27</f>
-        <v/>
+          <t>Courier to Zambia</t>
+        </is>
+      </c>
+      <c r="E44" s="34" t="n">
+        <v>0</v>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>order</t>
         </is>
       </c>
       <c r="G44" s="35">
         <f>E44*$D$4</f>
         <v/>
       </c>
-      <c r="H44" s="39">
-        <f>'Printed parts'!D27</f>
-        <v/>
+      <c r="H44" s="34" t="n">
+        <v>1</v>
       </c>
       <c r="I44" s="35">
         <f>G44+H44</f>
         <v/>
       </c>
       <c r="J44" s="34" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="K44" s="35">
         <f>IF(I44=0,0,ROUNDUP(I44/J44,0))</f>
         <v/>
       </c>
       <c r="L44" s="36" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="M44" s="37">
         <f>IF(Q44="Have already",0,K44*L44)</f>
@@ -4021,12 +3913,12 @@
       </c>
       <c r="N44" s="10" t="inlineStr">
         <is>
-          <t>Local / Bambu store</t>
+          <t>SparkFun</t>
         </is>
       </c>
       <c r="O44" s="15" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Import</t>
         </is>
       </c>
       <c r="P44" s="38" t="n"/>
@@ -4037,605 +3929,420 @@
       </c>
       <c r="R44" s="10" t="inlineStr">
         <is>
-          <t>Tyres only; about 25 g needed, so a small spool is enough.</t>
+          <t>Estimate. The courier may also bill VAT/duty on delivery (covered by the allowance below).</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>Packaging (optional)</t>
-        </is>
-      </c>
-      <c r="B45" s="8" t="n"/>
-      <c r="D45" s="8" t="n"/>
-      <c r="E45" s="8" t="n"/>
-      <c r="F45" s="8" t="n"/>
-      <c r="G45" s="8" t="n"/>
-      <c r="H45" s="8" t="n"/>
-      <c r="I45" s="8" t="n"/>
-      <c r="J45" s="8" t="n"/>
-      <c r="K45" s="8" t="n"/>
-      <c r="L45" s="8" t="n"/>
-      <c r="M45" s="8" t="n"/>
-      <c r="N45" s="8" t="n"/>
-      <c r="O45" s="8" t="n"/>
-      <c r="P45" s="8" t="n"/>
-      <c r="Q45" s="8" t="n"/>
-      <c r="R45" s="8" t="n"/>
-    </row>
-    <row r="46" ht="74" customHeight="1">
-      <c r="A46" s="9" t="n">
-        <v>32</v>
-      </c>
-      <c r="B46" s="10" t="inlineStr">
-        <is>
-          <t>Mailer box + printed quick-start guide</t>
-        </is>
-      </c>
-      <c r="C46" s="33" t="n"/>
-      <c r="D46" s="10" t="inlineStr">
-        <is>
-          <t>Design in mech/robot/packaging (273 × 203 × 83 mm outer)</t>
-        </is>
-      </c>
-      <c r="E46" s="34" t="n">
+      <c r="A45" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Shipping: AliExpress orders</t>
+        </is>
+      </c>
+      <c r="C45" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>All AliExpress parts</t>
+        </is>
+      </c>
+      <c r="E45" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>order</t>
+        </is>
+      </c>
+      <c r="G45" s="35">
+        <f>E45*$D$4</f>
+        <v/>
+      </c>
+      <c r="H45" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="F46" s="9" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="G46" s="35">
-        <f>E46*$D$4</f>
-        <v/>
-      </c>
-      <c r="H46" s="34" t="n">
+      <c r="I45" s="35">
+        <f>G45+H45</f>
+        <v/>
+      </c>
+      <c r="J45" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" s="35">
+        <f>IF(I45=0,0,ROUNDUP(I45/J45,0))</f>
+        <v/>
+      </c>
+      <c r="L45" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="M45" s="37">
+        <f>IF(Q45="Have already",0,K45*L45)</f>
+        <v/>
+      </c>
+      <c r="N45" s="10" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="O45" s="15" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="P45" s="38" t="n"/>
+      <c r="Q45" s="15" t="inlineStr">
+        <is>
+          <t>To buy</t>
+        </is>
+      </c>
+      <c r="R45" s="10" t="inlineStr">
+        <is>
+          <t>Estimate. Many stores ship free above a minimum order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>Tools (one-off; skip what you have)</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="n"/>
+      <c r="D46" s="8" t="n"/>
+      <c r="E46" s="8" t="n"/>
+      <c r="F46" s="8" t="n"/>
+      <c r="G46" s="8" t="n"/>
+      <c r="H46" s="8" t="n"/>
+      <c r="I46" s="8" t="n"/>
+      <c r="J46" s="8" t="n"/>
+      <c r="K46" s="8" t="n"/>
+      <c r="L46" s="8" t="n"/>
+      <c r="M46" s="8" t="n"/>
+      <c r="N46" s="8" t="n"/>
+      <c r="O46" s="8" t="n"/>
+      <c r="P46" s="8" t="n"/>
+      <c r="Q46" s="8" t="n"/>
+      <c r="R46" s="8" t="n"/>
+    </row>
+    <row r="47" ht="74" customHeight="1">
+      <c r="A47" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>Heat-set insert tips for the soldering iron</t>
+        </is>
+      </c>
+      <c r="C47" s="33" t="n"/>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>M2 and M3 tips to fit your iron</t>
+        </is>
+      </c>
+      <c r="E47" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="I46" s="35">
-        <f>G46+H46</f>
-        <v/>
-      </c>
-      <c r="J46" s="34" t="n">
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="G47" s="35">
+        <f>E47*$D$4</f>
+        <v/>
+      </c>
+      <c r="H47" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K46" s="35">
-        <f>IF(I46=0,0,ROUNDUP(I46/J46,0))</f>
-        <v/>
-      </c>
-      <c r="L46" s="36" t="n">
-        <v>2</v>
-      </c>
-      <c r="M46" s="37">
-        <f>IF(Q46="Have already",0,K46*L46)</f>
-        <v/>
-      </c>
-      <c r="N46" s="10" t="inlineStr">
-        <is>
-          <t>Local print shop</t>
-        </is>
-      </c>
-      <c r="O46" s="15" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="P46" s="38" t="n"/>
-      <c r="Q46" s="15" t="inlineStr">
-        <is>
-          <t>To buy</t>
-        </is>
-      </c>
-      <c r="R46" s="10" t="inlineStr">
-        <is>
-          <t>Estimate from the costing model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>Shipping (estimates; replace with the checkout price)</t>
-        </is>
-      </c>
-      <c r="B47" s="8" t="n"/>
-      <c r="D47" s="8" t="n"/>
-      <c r="E47" s="8" t="n"/>
-      <c r="F47" s="8" t="n"/>
-      <c r="G47" s="8" t="n"/>
-      <c r="H47" s="8" t="n"/>
-      <c r="I47" s="8" t="n"/>
-      <c r="J47" s="8" t="n"/>
-      <c r="K47" s="8" t="n"/>
-      <c r="L47" s="8" t="n"/>
-      <c r="M47" s="8" t="n"/>
-      <c r="N47" s="8" t="n"/>
-      <c r="O47" s="8" t="n"/>
-      <c r="P47" s="8" t="n"/>
-      <c r="Q47" s="8" t="n"/>
-      <c r="R47" s="8" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="n">
-        <v>33</v>
-      </c>
-      <c r="B48" s="10" t="inlineStr">
-        <is>
-          <t>Shipping: SparkFun order (motors)</t>
-        </is>
-      </c>
-      <c r="C48" s="40" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D48" s="10" t="inlineStr">
-        <is>
-          <t>Courier to Zambia</t>
-        </is>
-      </c>
-      <c r="E48" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" s="9" t="inlineStr">
-        <is>
-          <t>order</t>
-        </is>
-      </c>
-      <c r="G48" s="35">
-        <f>E48*$D$4</f>
-        <v/>
-      </c>
-      <c r="H48" s="34" t="n">
+      <c r="I47" s="35">
+        <f>G47+H47</f>
+        <v/>
+      </c>
+      <c r="J47" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="I48" s="35">
-        <f>G48+H48</f>
-        <v/>
-      </c>
-      <c r="J48" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="K48" s="35">
-        <f>IF(I48=0,0,ROUNDUP(I48/J48,0))</f>
-        <v/>
-      </c>
-      <c r="L48" s="36" t="n">
-        <v>50</v>
-      </c>
-      <c r="M48" s="37">
-        <f>IF(Q48="Have already",0,K48*L48)</f>
-        <v/>
-      </c>
-      <c r="N48" s="10" t="inlineStr">
-        <is>
-          <t>SparkFun</t>
-        </is>
-      </c>
-      <c r="O48" s="15" t="inlineStr">
+      <c r="K47" s="35">
+        <f>IF(I47=0,0,ROUNDUP(I47/J47,0))</f>
+        <v/>
+      </c>
+      <c r="L47" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="M47" s="37">
+        <f>IF(Q47="Have already",0,K47*L47)</f>
+        <v/>
+      </c>
+      <c r="N47" s="10" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="O47" s="15" t="inlineStr">
         <is>
           <t>Import</t>
         </is>
       </c>
-      <c r="P48" s="38" t="n"/>
-      <c r="Q48" s="15" t="inlineStr">
-        <is>
-          <t>To buy</t>
-        </is>
-      </c>
-      <c r="R48" s="10" t="inlineStr">
-        <is>
-          <t>Estimate. The courier may also bill VAT/duty on delivery (covered by the allowance below).</t>
-        </is>
-      </c>
-    </row>
+      <c r="P47" s="38" t="n"/>
+      <c r="Q47" s="15" t="inlineStr">
+        <is>
+          <t>Have already</t>
+        </is>
+      </c>
+      <c r="R47" s="10" t="inlineStr">
+        <is>
+          <t>Set to 'To buy' if your iron has none. Also used: soldering iron, multimeter (to match the cells).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
     <row r="49">
-      <c r="A49" s="9" t="n">
-        <v>34</v>
-      </c>
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t>Shipping: AliExpress orders</t>
-        </is>
-      </c>
-      <c r="C49" s="40" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D49" s="10" t="inlineStr">
-        <is>
-          <t>All AliExpress parts</t>
-        </is>
-      </c>
-      <c r="E49" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F49" s="9" t="inlineStr">
-        <is>
-          <t>order</t>
-        </is>
-      </c>
-      <c r="G49" s="35">
-        <f>E49*$D$4</f>
-        <v/>
-      </c>
-      <c r="H49" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="I49" s="35">
-        <f>G49+H49</f>
-        <v/>
-      </c>
-      <c r="J49" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="K49" s="35">
-        <f>IF(I49=0,0,ROUNDUP(I49/J49,0))</f>
-        <v/>
-      </c>
-      <c r="L49" s="36" t="n">
-        <v>10</v>
-      </c>
-      <c r="M49" s="37">
-        <f>IF(Q49="Have already",0,K49*L49)</f>
-        <v/>
-      </c>
-      <c r="N49" s="10" t="inlineStr">
-        <is>
-          <t>AliExpress</t>
-        </is>
-      </c>
-      <c r="O49" s="15" t="inlineStr">
-        <is>
-          <t>Import</t>
-        </is>
-      </c>
-      <c r="P49" s="38" t="n"/>
-      <c r="Q49" s="15" t="inlineStr">
-        <is>
-          <t>To buy</t>
-        </is>
-      </c>
-      <c r="R49" s="10" t="inlineStr">
-        <is>
-          <t>Estimate. Many stores ship free above a minimum order.</t>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>Summary</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>Tools (one-off; skip what you have)</t>
-        </is>
-      </c>
-      <c r="B50" s="8" t="n"/>
-      <c r="D50" s="8" t="n"/>
-      <c r="E50" s="8" t="n"/>
-      <c r="F50" s="8" t="n"/>
-      <c r="G50" s="8" t="n"/>
-      <c r="H50" s="8" t="n"/>
-      <c r="I50" s="8" t="n"/>
-      <c r="J50" s="8" t="n"/>
-      <c r="K50" s="8" t="n"/>
-      <c r="L50" s="8" t="n"/>
-      <c r="M50" s="8" t="n"/>
-      <c r="N50" s="8" t="n"/>
-      <c r="O50" s="8" t="n"/>
-      <c r="P50" s="8" t="n"/>
-      <c r="Q50" s="8" t="n"/>
-      <c r="R50" s="8" t="n"/>
-    </row>
-    <row r="51" ht="74" customHeight="1">
-      <c r="A51" s="9" t="n">
-        <v>35</v>
-      </c>
-      <c r="B51" s="10" t="inlineStr">
-        <is>
-          <t>Heat-set insert tips for the soldering iron</t>
-        </is>
-      </c>
-      <c r="C51" s="33" t="n"/>
-      <c r="D51" s="10" t="inlineStr">
-        <is>
-          <t>M2 and M3 tips to fit your iron</t>
-        </is>
-      </c>
-      <c r="E51" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>set</t>
-        </is>
-      </c>
-      <c r="G51" s="35">
-        <f>E51*$D$4</f>
-        <v/>
-      </c>
-      <c r="H51" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="I51" s="35">
-        <f>G51+H51</f>
-        <v/>
-      </c>
-      <c r="J51" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="K51" s="35">
-        <f>IF(I51=0,0,ROUNDUP(I51/J51,0))</f>
-        <v/>
-      </c>
-      <c r="L51" s="36" t="n">
-        <v>5</v>
-      </c>
-      <c r="M51" s="37">
-        <f>IF(Q51="Have already",0,K51*L51)</f>
-        <v/>
-      </c>
-      <c r="N51" s="10" t="inlineStr">
-        <is>
-          <t>AliExpress</t>
-        </is>
-      </c>
-      <c r="O51" s="15" t="inlineStr">
-        <is>
-          <t>Import</t>
-        </is>
-      </c>
-      <c r="P51" s="38" t="n"/>
-      <c r="Q51" s="15" t="inlineStr">
-        <is>
-          <t>Have already</t>
-        </is>
-      </c>
-      <c r="R51" s="10" t="inlineStr">
-        <is>
-          <t>Set to 'To buy' if your iron has none. Also used: soldering iron, multimeter (to match the cells).</t>
-        </is>
-      </c>
-    </row>
-    <row r="52"/>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Estimated cost, all lines</t>
+        </is>
+      </c>
+      <c r="M50" s="41">
+        <f>SUM(M8:M47)</f>
+        <v/>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>Everything above at the estimated prices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which: controller boards (PCBWay)</t>
+        </is>
+      </c>
+      <c r="M51" s="42">
+        <f>M9</f>
+        <v/>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>Already quoted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which: everything else</t>
+        </is>
+      </c>
+      <c r="M52" s="42">
+        <f>M50-M51</f>
+        <v/>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>What this list still has to buy.</t>
+        </is>
+      </c>
+    </row>
     <row r="53">
-      <c r="B53" s="18" t="inlineStr">
-        <is>
-          <t>Summary</t>
+      <c r="B53" s="20" t="inlineStr">
+        <is>
+          <t>Import VAT + duty allowance</t>
+        </is>
+      </c>
+      <c r="M53" s="42">
+        <f>SUMIF(O8:O47,"Import",M8:M47)*$D$5</f>
+        <v/>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>Allowance rate (C5) × lines marked Import.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Estimated cost, all lines</t>
-        </is>
-      </c>
-      <c r="M54" s="41">
-        <f>SUM(M8:M51)</f>
-        <v/>
-      </c>
-      <c r="N54" s="2" t="inlineStr">
-        <is>
-          <t>Everything above at the estimated prices.</t>
-        </is>
-      </c>
+          <t>Estimated total, landed</t>
+        </is>
+      </c>
+      <c r="M54" s="43">
+        <f>M50+M53</f>
+        <v/>
+      </c>
+      <c r="N54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="B55" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  of which: controller boards (PCBWay)</t>
-        </is>
-      </c>
-      <c r="M55" s="42">
-        <f>M9</f>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Per robot</t>
+        </is>
+      </c>
+      <c r="M55" s="43">
+        <f>IF($D$4=0,0,M54/$D$4)</f>
         <v/>
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>Already quoted.</t>
+          <t>Before labour (about 1.5 h per robot to assemble and test).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  of which: everything else</t>
+          <t>Actually paid so far</t>
         </is>
       </c>
       <c r="M56" s="42">
-        <f>M54-M55</f>
+        <f>SUM(P8:P47)</f>
         <v/>
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>What this list still has to buy.</t>
+          <t>From the yellow 'Actual paid' column.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="20" t="inlineStr">
         <is>
-          <t>Import VAT + duty allowance</t>
-        </is>
-      </c>
-      <c r="M57" s="42">
-        <f>SUMIF(O8:O51,"Import",M8:M51)*$D$5</f>
-        <v/>
-      </c>
-      <c r="N57" s="2" t="inlineStr">
-        <is>
-          <t>Allowance rate (C5) × lines marked Import.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>Estimated total, landed</t>
-        </is>
-      </c>
-      <c r="M58" s="43">
-        <f>M54+M57</f>
-        <v/>
-      </c>
-      <c r="N58" s="2" t="inlineStr"/>
-    </row>
+          <t>Lines still 'To buy'</t>
+        </is>
+      </c>
+      <c r="M57" s="44">
+        <f>COUNTIF(Q8:Q47,"To buy")</f>
+        <v/>
+      </c>
+      <c r="N57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58"/>
     <row r="59">
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>Per robot</t>
-        </is>
-      </c>
-      <c r="M59" s="43">
-        <f>IF($D$4=0,0,M58/$D$4)</f>
-        <v/>
-      </c>
-      <c r="N59" s="2" t="inlineStr">
-        <is>
-          <t>Before labour (about 1.5 h per robot to assemble and test).</t>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>Cost by section (estimate)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="20" t="inlineStr">
         <is>
-          <t>Actually paid so far</t>
+          <t>Controller board (on order at PCBWay)</t>
         </is>
       </c>
       <c r="M60" s="42">
-        <f>SUM(P8:P51)</f>
-        <v/>
-      </c>
-      <c r="N60" s="2" t="inlineStr">
-        <is>
-          <t>From the yellow 'Actual paid' column.</t>
-        </is>
+        <f>SUM(M9:M9)</f>
+        <v/>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="20" t="inlineStr">
         <is>
-          <t>Lines still 'To buy'</t>
-        </is>
-      </c>
-      <c r="M61" s="44">
-        <f>COUNTIF(Q8:Q51,"To buy")</f>
-        <v/>
-      </c>
-      <c r="N61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62"/>
+          <t>Motors, sensors and servos</t>
+        </is>
+      </c>
+      <c r="M61" s="42">
+        <f>SUM(M11:M14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="20" t="inlineStr">
+        <is>
+          <t>Battery and power</t>
+        </is>
+      </c>
+      <c r="M62" s="42">
+        <f>SUM(M16:M18)</f>
+        <v/>
+      </c>
+    </row>
     <row r="63">
-      <c r="B63" s="18" t="inlineStr">
-        <is>
-          <t>Cost by section (estimate)</t>
-        </is>
+      <c r="B63" s="20" t="inlineStr">
+        <is>
+          <t>Cables</t>
+        </is>
+      </c>
+      <c r="M63" s="42">
+        <f>SUM(M20:M21)</f>
+        <v/>
       </c>
     </row>
     <row r="64">
       <c r="B64" s="20" t="inlineStr">
         <is>
-          <t>Controller board (on order at PCBWay)</t>
+          <t>Screws, inserts and small hardware (with the arm and one bus clip)</t>
         </is>
       </c>
       <c r="M64" s="42">
-        <f>SUM(M9:M9)</f>
+        <f>SUM(M23:M35)</f>
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="B65" s="20" t="inlineStr">
         <is>
-          <t>Motors, sensors and servos</t>
+          <t>3D printing filament (grams, from the Printed parts sheet)</t>
         </is>
       </c>
       <c r="M65" s="42">
-        <f>SUM(M11:M15)</f>
+        <f>SUM(M37:M40)</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="B66" s="20" t="inlineStr">
         <is>
-          <t>Battery and power</t>
+          <t>Packaging (optional)</t>
         </is>
       </c>
       <c r="M66" s="42">
-        <f>SUM(M17:M21)</f>
+        <f>SUM(M42:M42)</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="20" t="inlineStr">
         <is>
-          <t>Cables</t>
+          <t>Shipping (estimates; replace with the checkout price)</t>
         </is>
       </c>
       <c r="M67" s="42">
-        <f>SUM(M23:M25)</f>
+        <f>SUM(M44:M45)</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="B68" s="20" t="inlineStr">
         <is>
-          <t>Screws, inserts and small hardware (with the arm and one bus clip)</t>
+          <t>Tools (one-off; skip what you have)</t>
         </is>
       </c>
       <c r="M68" s="42">
-        <f>SUM(M27:M39)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="20" t="inlineStr">
-        <is>
-          <t>3D printing filament (grams, from the Printed parts sheet)</t>
-        </is>
-      </c>
-      <c r="M69" s="42">
-        <f>SUM(M41:M44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="20" t="inlineStr">
-        <is>
-          <t>Packaging (optional)</t>
-        </is>
-      </c>
-      <c r="M70" s="42">
-        <f>SUM(M46:M46)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="20" t="inlineStr">
-        <is>
-          <t>Shipping (estimates; replace with the checkout price)</t>
-        </is>
-      </c>
-      <c r="M71" s="42">
-        <f>SUM(M48:M49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" s="20" t="inlineStr">
-        <is>
-          <t>Tools (one-off; skip what you have)</t>
-        </is>
-      </c>
-      <c r="M72" s="42">
-        <f>SUM(M51:M51)</f>
-        <v/>
-      </c>
-    </row>
+        <f>SUM(M47:M47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
   </sheetData>
-  <autoFilter ref="A7:R51"/>
-  <conditionalFormatting sqref="Q8:Q51">
+  <autoFilter ref="A7:R47"/>
+  <conditionalFormatting sqref="Q8:Q47">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Received"</formula>
     </cfRule>
@@ -4650,10 +4357,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="Q8:Q51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Q8:Q47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To buy,Quoted,Ordered,Received,Have already"</formula1>
     </dataValidation>
-    <dataValidation sqref="O8:O51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="O8:O47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Import,Local"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5533,7 +5240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -5558,7 +5265,7 @@
     <row r="5">
       <c r="A5" s="32" t="inlineStr">
         <is>
-          <t>Change 'Robots to build' (Component list, C4) and every quantity and total updates. The filament grams follow the Printed parts sheet.</t>
+          <t>Change 'Robots to build' (Component list, D4) and every quantity and total updates. The filament grams follow the Printed parts sheet.</t>
         </is>
       </c>
     </row>
@@ -5629,7 +5336,7 @@
     <row r="16">
       <c r="A16" s="32" t="inlineStr">
         <is>
-          <t>4. Battery: holder wired in parallel (1S3P), never in series. Add a 1S protection board: the controller has no low-battery cut-off.</t>
+          <t>4. Battery: holder wired in parallel (1S3P), never in series. No protection board (Fred, 2026-10-12). The controller guards against a reversed pack, a 2S/3S pack and over-charging, but has no low-battery cut-off: switch robots off after use.</t>
         </is>
       </c>
     </row>
@@ -5651,7 +5358,7 @@
     <row r="20">
       <c r="A20" s="32" t="inlineStr">
         <is>
-          <t>Labour (about 1.5 h per robot), printer time (about 13 h per robot), tools you already have, and any duty above the allowance in C5.</t>
+          <t>Labour (about 1.5 h per robot), printer time (about 13 h per robot), tools you already have, and any duty above the allowance in D5.</t>
         </is>
       </c>
     </row>
@@ -5695,6 +5402,13 @@
       <c r="A27" s="32" t="inlineStr">
         <is>
           <t>Connector facts (J403 3.3 V, J404 analog, XT30 male on the board): docs/RoboCore_V2_spec.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-12: both arm servos are MG90S (one line). Removed at Fred's request: SG90, 1S protection board, heat-shrink, USB-C cable. Fasteners follow the rev 5 robot design; the notes column says where each one goes.</t>
         </is>
       </c>
     </row>

</xml_diff>